<commit_message>
Update v3.3 ledger 2026-10-05
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7090,7 +7090,9 @@
       <c r="C47" s="119" t="n">
         <v>104.006950258</v>
       </c>
-      <c r="D47" s="84" t="n"/>
+      <c r="D47" s="84" t="n">
+        <v>756.2</v>
+      </c>
       <c r="E47" s="84">
         <f>IF(D47="","",D47*C47)</f>
         <v/>
@@ -7101,6 +7103,9 @@
       </c>
       <c r="G47" s="127" t="n">
         <v>450.617228933</v>
+      </c>
+      <c r="H47" t="n">
+        <v>83.12</v>
       </c>
       <c r="I47" s="84">
         <f>IF(H47="","",H47*G47)</f>
@@ -7192,7 +7197,9 @@
         <f>IF(OR(AE47="",B47="",B47=0),"",AE47/B47)</f>
         <v/>
       </c>
-      <c r="AG47" s="125" t="n"/>
+      <c r="AG47" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH47" s="126" t="n"/>
       <c r="AI47" s="126" t="n"/>
       <c r="AJ47" s="126" t="n"/>
@@ -7232,13 +7239,45 @@
         <f>IF(B48="","",F48+J48*3)</f>
         <v/>
       </c>
-      <c r="O48" s="122" t="n"/>
-      <c r="P48" s="83" t="n"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>1.61x</t>
+        </is>
+      </c>
+      <c r="O48" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P48" s="83" t="n">
+        <v>0.55</v>
+      </c>
       <c r="Q48" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R48" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S48" t="n">
+        <v>125</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V48" s="123">
         <f>IF(OR(B48="",B47=""),"",B48/B47-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-06
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7104,7 +7104,7 @@
       <c r="G47" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="67" t="n">
         <v>83.12</v>
       </c>
       <c r="I47" s="84">
@@ -7215,7 +7215,9 @@
       <c r="C48" s="119" t="n">
         <v>104.006950258</v>
       </c>
-      <c r="D48" s="84" t="n"/>
+      <c r="D48" s="84" t="n">
+        <v>759.66</v>
+      </c>
       <c r="E48" s="84">
         <f>IF(D48="","",D48*C48)</f>
         <v/>
@@ -7227,6 +7229,9 @@
       <c r="G48" s="127" t="n">
         <v>450.617228933</v>
       </c>
+      <c r="H48" t="n">
+        <v>84.25</v>
+      </c>
       <c r="I48" s="84">
         <f>IF(H48="","",H48*G48)</f>
         <v/>
@@ -7239,17 +7244,17 @@
         <f>IF(B48="","",F48+J48*3)</f>
         <v/>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M48" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="N48" s="67" t="inlineStr">
         <is>
           <t>1.61x</t>
         </is>
@@ -7266,15 +7271,15 @@
       <c r="R48" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S48" t="n">
+      <c r="S48" s="67" t="n">
         <v>125</v>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T48" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U48" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7317,7 +7322,9 @@
         <f>IF(OR(AE48="",B48="",B48=0),"",AE48/B48)</f>
         <v/>
       </c>
-      <c r="AG48" s="125" t="n"/>
+      <c r="AG48" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH48" s="126" t="n"/>
       <c r="AI48" s="126" t="n"/>
       <c r="AJ48" s="126" t="n"/>
@@ -7357,13 +7364,45 @@
         <f>IF(B49="","",F49+J49*3)</f>
         <v/>
       </c>
-      <c r="O49" s="122" t="n"/>
-      <c r="P49" s="83" t="n"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>1.60x</t>
+        </is>
+      </c>
+      <c r="O49" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P49" s="83" t="n">
+        <v>0.53</v>
+      </c>
       <c r="Q49" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R49" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S49" t="n">
+        <v>126</v>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V49" s="123">
         <f>IF(OR(B49="",B48=""),"",B49/B48-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-07
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7229,7 +7229,7 @@
       <c r="G48" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H48" t="n">
+      <c r="H48" s="67" t="n">
         <v>84.25</v>
       </c>
       <c r="I48" s="84">
@@ -7340,7 +7340,9 @@
       <c r="C49" s="119" t="n">
         <v>104.006950258</v>
       </c>
-      <c r="D49" s="84" t="n"/>
+      <c r="D49" s="84" t="n">
+        <v>757.73</v>
+      </c>
       <c r="E49" s="84">
         <f>IF(D49="","",D49*C49)</f>
         <v/>
@@ -7352,6 +7354,9 @@
       <c r="G49" s="127" t="n">
         <v>450.617228933</v>
       </c>
+      <c r="H49" t="n">
+        <v>83.62</v>
+      </c>
       <c r="I49" s="84">
         <f>IF(H49="","",H49*G49)</f>
         <v/>
@@ -7364,17 +7369,17 @@
         <f>IF(B49="","",F49+J49*3)</f>
         <v/>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M49" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="N49" s="67" t="inlineStr">
         <is>
           <t>1.60x</t>
         </is>
@@ -7391,15 +7396,15 @@
       <c r="R49" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S49" t="n">
+      <c r="S49" s="67" t="n">
         <v>126</v>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="T49" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="U49" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7442,7 +7447,9 @@
         <f>IF(OR(AE49="",B49="",B49=0),"",AE49/B49)</f>
         <v/>
       </c>
-      <c r="AG49" s="125" t="n"/>
+      <c r="AG49" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH49" s="126" t="n"/>
       <c r="AI49" s="126" t="n"/>
       <c r="AJ49" s="126" t="n"/>
@@ -7478,13 +7485,45 @@
         <f>IF(B50="","",F50+J50*3)</f>
         <v/>
       </c>
-      <c r="O50" s="122" t="n"/>
-      <c r="P50" s="83" t="n"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>1.60x</t>
+        </is>
+      </c>
+      <c r="O50" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P50" s="83" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="Q50" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R50" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S50" t="n">
+        <v>127</v>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V50" s="123">
         <f>IF(OR(B50="",B49=""),"",B50/B49-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-08
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7354,7 +7354,7 @@
       <c r="G49" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H49" t="n">
+      <c r="H49" s="67" t="n">
         <v>83.62</v>
       </c>
       <c r="I49" s="84">
@@ -7462,8 +7462,12 @@
         <f>IF(AND(E50="",I50="",AE50="",AG50=""),"",SUM(E50,I50,AE50,AG50))</f>
         <v/>
       </c>
-      <c r="C50" s="119" t="n"/>
-      <c r="D50" s="84" t="n"/>
+      <c r="C50" s="119" t="n">
+        <v>104.006950258</v>
+      </c>
+      <c r="D50" s="84" t="n">
+        <v>747.58</v>
+      </c>
       <c r="E50" s="84">
         <f>IF(D50="","",D50*C50)</f>
         <v/>
@@ -7472,7 +7476,12 @@
         <f>IF(B50="","",E50/B50)</f>
         <v/>
       </c>
-      <c r="G50" s="127" t="n"/>
+      <c r="G50" s="127" t="n">
+        <v>450.617228933</v>
+      </c>
+      <c r="H50" t="n">
+        <v>80.23</v>
+      </c>
       <c r="I50" s="84">
         <f>IF(H50="","",H50*G50)</f>
         <v/>
@@ -7485,17 +7494,17 @@
         <f>IF(B50="","",F50+J50*3)</f>
         <v/>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L50" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M50" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="N50" s="67" t="inlineStr">
         <is>
           <t>1.60x</t>
         </is>
@@ -7512,15 +7521,15 @@
       <c r="R50" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S50" t="n">
+      <c r="S50" s="67" t="n">
         <v>127</v>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="T50" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="U50" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7563,7 +7572,9 @@
         <f>IF(OR(AE50="",B50="",B50=0),"",AE50/B50)</f>
         <v/>
       </c>
-      <c r="AG50" s="125" t="n"/>
+      <c r="AG50" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH50" s="126" t="n"/>
       <c r="AI50" s="126" t="n"/>
       <c r="AJ50" s="126" t="n"/>
@@ -7599,13 +7610,45 @@
         <f>IF(B51="","",F51+J51*3)</f>
         <v/>
       </c>
-      <c r="O51" s="122" t="n"/>
-      <c r="P51" s="83" t="n"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>1.57x</t>
+        </is>
+      </c>
+      <c r="O51" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P51" s="83" t="n">
+        <v>0.59</v>
+      </c>
       <c r="Q51" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R51" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S51" t="n">
+        <v>128</v>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V51" s="123">
         <f>IF(OR(B51="",B50=""),"",B51/B50-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-09
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7479,7 +7479,7 @@
       <c r="G50" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H50" t="n">
+      <c r="H50" s="67" t="n">
         <v>80.23</v>
       </c>
       <c r="I50" s="84">
@@ -7587,8 +7587,12 @@
         <f>IF(AND(E51="",I51="",AE51="",AG51=""),"",SUM(E51,I51,AE51,AG51))</f>
         <v/>
       </c>
-      <c r="C51" s="119" t="n"/>
-      <c r="D51" s="84" t="n"/>
+      <c r="C51" s="119" t="n">
+        <v>104.006950258</v>
+      </c>
+      <c r="D51" s="84" t="n">
+        <v>751.27</v>
+      </c>
       <c r="E51" s="84">
         <f>IF(D51="","",D51*C51)</f>
         <v/>
@@ -7597,7 +7601,12 @@
         <f>IF(B51="","",E51/B51)</f>
         <v/>
       </c>
-      <c r="G51" s="127" t="n"/>
+      <c r="G51" s="127" t="n">
+        <v>450.617228933</v>
+      </c>
+      <c r="H51" t="n">
+        <v>81.28</v>
+      </c>
       <c r="I51" s="84">
         <f>IF(H51="","",H51*G51)</f>
         <v/>
@@ -7610,17 +7619,17 @@
         <f>IF(B51="","",F51+J51*3)</f>
         <v/>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="L51" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="M51" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="N51" s="67" t="inlineStr">
         <is>
           <t>1.57x</t>
         </is>
@@ -7637,15 +7646,15 @@
       <c r="R51" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S51" t="n">
+      <c r="S51" s="67" t="n">
         <v>128</v>
       </c>
-      <c r="T51" t="inlineStr">
+      <c r="T51" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="U51" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7688,7 +7697,9 @@
         <f>IF(OR(AE51="",B51="",B51=0),"",AE51/B51)</f>
         <v/>
       </c>
-      <c r="AG51" s="125" t="n"/>
+      <c r="AG51" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH51" s="126" t="n"/>
       <c r="AI51" s="126" t="n"/>
       <c r="AJ51" s="126" t="n"/>
@@ -7724,13 +7735,45 @@
         <f>IF(B52="","",F52+J52*3)</f>
         <v/>
       </c>
-      <c r="O52" s="122" t="n"/>
-      <c r="P52" s="83" t="n"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>1.60x</t>
+        </is>
+      </c>
+      <c r="O52" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P52" s="83" t="n">
+        <v>0.53</v>
+      </c>
       <c r="Q52" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R52" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S52" t="n">
+        <v>129</v>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V52" s="123">
         <f>IF(OR(B52="",B51=""),"",B52/B51-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-12
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7604,7 +7604,7 @@
       <c r="G51" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H51" t="n">
+      <c r="H51" s="67" t="n">
         <v>81.28</v>
       </c>
       <c r="I51" s="84">
@@ -7712,8 +7712,12 @@
         <f>IF(AND(E52="",I52="",AE52="",AG52=""),"",SUM(E52,I52,AE52,AG52))</f>
         <v/>
       </c>
-      <c r="C52" s="119" t="n"/>
-      <c r="D52" s="84" t="n"/>
+      <c r="C52" s="119" t="n">
+        <v>104.006950258</v>
+      </c>
+      <c r="D52" s="84" t="n">
+        <v>746.04</v>
+      </c>
       <c r="E52" s="84">
         <f>IF(D52="","",D52*C52)</f>
         <v/>
@@ -7722,7 +7726,12 @@
         <f>IF(B52="","",E52/B52)</f>
         <v/>
       </c>
-      <c r="G52" s="127" t="n"/>
+      <c r="G52" s="127" t="n">
+        <v>450.617228933</v>
+      </c>
+      <c r="H52" t="n">
+        <v>79.61</v>
+      </c>
       <c r="I52" s="84">
         <f>IF(H52="","",H52*G52)</f>
         <v/>
@@ -7735,17 +7744,17 @@
         <f>IF(B52="","",F52+J52*3)</f>
         <v/>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L52" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M52" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="N52" s="67" t="inlineStr">
         <is>
           <t>1.60x</t>
         </is>
@@ -7762,15 +7771,15 @@
       <c r="R52" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S52" t="n">
+      <c r="S52" s="67" t="n">
         <v>129</v>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="T52" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="U52" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7813,7 +7822,9 @@
         <f>IF(OR(AE52="",B52="",B52=0),"",AE52/B52)</f>
         <v/>
       </c>
-      <c r="AG52" s="125" t="n"/>
+      <c r="AG52" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH52" s="126" t="n"/>
       <c r="AI52" s="126" t="n"/>
       <c r="AJ52" s="126" t="n"/>
@@ -7849,13 +7860,45 @@
         <f>IF(B53="","",F53+J53*3)</f>
         <v/>
       </c>
-      <c r="O53" s="122" t="n"/>
-      <c r="P53" s="83" t="n"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>1.60x</t>
+        </is>
+      </c>
+      <c r="O53" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P53" s="83" t="n">
+        <v>0.54</v>
+      </c>
       <c r="Q53" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R53" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S53" t="n">
+        <v>130</v>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V53" s="123">
         <f>IF(OR(B53="",B52=""),"",B53/B52-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-13
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7729,7 +7729,7 @@
       <c r="G52" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H52" t="n">
+      <c r="H52" s="67" t="n">
         <v>79.61</v>
       </c>
       <c r="I52" s="84">
@@ -7837,8 +7837,12 @@
         <f>IF(AND(E53="",I53="",AE53="",AG53=""),"",SUM(E53,I53,AE53,AG53))</f>
         <v/>
       </c>
-      <c r="C53" s="119" t="n"/>
-      <c r="D53" s="84" t="n"/>
+      <c r="C53" s="119" t="n">
+        <v>104.006950258</v>
+      </c>
+      <c r="D53" s="84" t="n">
+        <v>743.5700000000001</v>
+      </c>
       <c r="E53" s="84">
         <f>IF(D53="","",D53*C53)</f>
         <v/>
@@ -7847,7 +7851,12 @@
         <f>IF(B53="","",E53/B53)</f>
         <v/>
       </c>
-      <c r="G53" s="127" t="n"/>
+      <c r="G53" s="127" t="n">
+        <v>450.617228933</v>
+      </c>
+      <c r="H53" t="n">
+        <v>78.81</v>
+      </c>
       <c r="I53" s="84">
         <f>IF(H53="","",H53*G53)</f>
         <v/>
@@ -7860,17 +7869,17 @@
         <f>IF(B53="","",F53+J53*3)</f>
         <v/>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="L53" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="M53" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="N53" s="67" t="inlineStr">
         <is>
           <t>1.60x</t>
         </is>
@@ -7887,15 +7896,15 @@
       <c r="R53" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S53" t="n">
+      <c r="S53" s="67" t="n">
         <v>130</v>
       </c>
-      <c r="T53" t="inlineStr">
+      <c r="T53" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="U53" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7938,7 +7947,9 @@
         <f>IF(OR(AE53="",B53="",B53=0),"",AE53/B53)</f>
         <v/>
       </c>
-      <c r="AG53" s="125" t="n"/>
+      <c r="AG53" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH53" s="126" t="n"/>
       <c r="AI53" s="126" t="n"/>
       <c r="AJ53" s="126" t="n"/>
@@ -7974,13 +7985,45 @@
         <f>IF(B54="","",F54+J54*3)</f>
         <v/>
       </c>
-      <c r="O54" s="122" t="n"/>
-      <c r="P54" s="83" t="n"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>1.63x</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>1.62x</t>
+        </is>
+      </c>
+      <c r="O54" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P54" s="83" t="n">
+        <v>0.54</v>
+      </c>
       <c r="Q54" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R54" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S54" t="n">
+        <v>131</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V54" s="123">
         <f>IF(OR(B54="",B53=""),"",B54/B53-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-14
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7854,7 +7854,7 @@
       <c r="G53" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H53" t="n">
+      <c r="H53" s="67" t="n">
         <v>78.81</v>
       </c>
       <c r="I53" s="84">
@@ -7962,8 +7962,12 @@
         <f>IF(AND(E54="",I54="",AE54="",AG54=""),"",SUM(E54,I54,AE54,AG54))</f>
         <v/>
       </c>
-      <c r="C54" s="119" t="n"/>
-      <c r="D54" s="84" t="n"/>
+      <c r="C54" s="119" t="n">
+        <v>104.006950258</v>
+      </c>
+      <c r="D54" s="84" t="n">
+        <v>728.95</v>
+      </c>
       <c r="E54" s="84">
         <f>IF(D54="","",D54*C54)</f>
         <v/>
@@ -7972,7 +7976,12 @@
         <f>IF(B54="","",E54/B54)</f>
         <v/>
       </c>
-      <c r="G54" s="127" t="n"/>
+      <c r="G54" s="127" t="n">
+        <v>450.617228933</v>
+      </c>
+      <c r="H54" t="n">
+        <v>74.12</v>
+      </c>
       <c r="I54" s="84">
         <f>IF(H54="","",H54*G54)</f>
         <v/>
@@ -7985,17 +7994,17 @@
         <f>IF(B54="","",F54+J54*3)</f>
         <v/>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L54" s="67" t="inlineStr">
         <is>
           <t>1.63x</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="M54" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="N54" s="67" t="inlineStr">
         <is>
           <t>1.62x</t>
         </is>
@@ -8012,15 +8021,15 @@
       <c r="R54" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S54" t="n">
+      <c r="S54" s="67" t="n">
         <v>131</v>
       </c>
-      <c r="T54" t="inlineStr">
+      <c r="T54" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="U54" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8063,7 +8072,9 @@
         <f>IF(OR(AE54="",B54="",B54=0),"",AE54/B54)</f>
         <v/>
       </c>
-      <c r="AG54" s="125" t="n"/>
+      <c r="AG54" s="125" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AH54" s="126" t="n"/>
       <c r="AI54" s="126" t="n"/>
       <c r="AJ54" s="126" t="n"/>
@@ -8099,13 +8110,45 @@
         <f>IF(B55="","",F55+J55*3)</f>
         <v/>
       </c>
-      <c r="O55" s="122" t="n"/>
-      <c r="P55" s="83" t="n"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>1.46x</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>REBALANCE — 68.51% QQQ / 31.49% TQQQ → 76.83% QQQ / 23.17% TQQQ</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>1.46x</t>
+        </is>
+      </c>
+      <c r="O55" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P55" s="83" t="n">
+        <v>0.59</v>
+      </c>
       <c r="Q55" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R55" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S55" t="n">
+        <v>132</v>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V55" s="123">
         <f>IF(OR(B55="",B54=""),"",B55/B54-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-15
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -7979,7 +7979,7 @@
       <c r="G54" s="127" t="n">
         <v>450.617228933</v>
       </c>
-      <c r="H54" t="n">
+      <c r="H54" s="67" t="n">
         <v>74.12</v>
       </c>
       <c r="I54" s="84">
@@ -8087,8 +8087,12 @@
         <f>IF(AND(E55="",I55="",AE55="",AG55=""),"",SUM(E55,I55,AE55,AG55))</f>
         <v/>
       </c>
-      <c r="C55" s="119" t="n"/>
-      <c r="D55" s="84" t="n"/>
+      <c r="C55" s="119" t="n">
+        <v>114.784904705</v>
+      </c>
+      <c r="D55" s="84" t="n">
+        <v>728</v>
+      </c>
       <c r="E55" s="84">
         <f>IF(D55="","",D55*C55)</f>
         <v/>
@@ -8097,7 +8101,12 @@
         <f>IF(B55="","",E55/B55)</f>
         <v/>
       </c>
-      <c r="G55" s="127" t="n"/>
+      <c r="G55" s="127" t="n">
+        <v>340.980401015</v>
+      </c>
+      <c r="H55" t="n">
+        <v>73.81999999999999</v>
+      </c>
       <c r="I55" s="84">
         <f>IF(H55="","",H55*G55)</f>
         <v/>
@@ -8110,17 +8119,17 @@
         <f>IF(B55="","",F55+J55*3)</f>
         <v/>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="L55" s="67" t="inlineStr">
         <is>
           <t>1.46x</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="M55" s="67" t="inlineStr">
         <is>
           <t>REBALANCE — 68.51% QQQ / 31.49% TQQQ → 76.83% QQQ / 23.17% TQQQ</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
+      <c r="N55" s="67" t="inlineStr">
         <is>
           <t>1.46x</t>
         </is>
@@ -8137,15 +8146,15 @@
       <c r="R55" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S55" t="n">
+      <c r="S55" s="67" t="n">
         <v>132</v>
       </c>
-      <c r="T55" t="inlineStr">
+      <c r="T55" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="U55" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8188,8 +8197,14 @@
         <f>IF(OR(AE55="",B55="",B55=0),"",AE55/B55)</f>
         <v/>
       </c>
-      <c r="AG55" s="125" t="n"/>
-      <c r="AH55" s="126" t="n"/>
+      <c r="AG55" s="125" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="AH55" s="126" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="AI55" s="126" t="n"/>
       <c r="AJ55" s="126" t="n"/>
     </row>
@@ -8224,13 +8239,45 @@
         <f>IF(B56="","",F56+J56*3)</f>
         <v/>
       </c>
-      <c r="O56" s="122" t="n"/>
-      <c r="P56" s="83" t="n"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>1.57x</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>REBALANCE — 76.83% QQQ / 23.17% TQQQ → 71.66% QQQ / 28.34% TQQQ</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>1.57x</t>
+        </is>
+      </c>
+      <c r="O56" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P56" s="83" t="n">
+        <v>0.54</v>
+      </c>
       <c r="Q56" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R56" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S56" t="n">
+        <v>133</v>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V56" s="123">
         <f>IF(OR(B56="",B55=""),"",B56/B55-1)</f>
@@ -15374,38 +15421,70 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="68">
-      <c r="A25" s="126" t="n"/>
-      <c r="B25" s="126" t="n"/>
-      <c r="C25" s="126" t="n"/>
-      <c r="D25" s="126" t="n"/>
+      <c r="A25" s="131" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B25" s="73" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C25" s="73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="D25" s="73" t="n">
+        <v>109.636827918</v>
+      </c>
       <c r="E25" s="78">
         <f>IF(OR(D25="",G25=""),"",D25*G25)</f>
         <v/>
       </c>
-      <c r="F25" s="125" t="n"/>
-      <c r="G25" s="125" t="n"/>
+      <c r="F25" s="78" t="n">
+        <v>70.485</v>
+      </c>
+      <c r="G25" s="78" t="n">
+        <v>70.49529</v>
+      </c>
       <c r="H25" s="135">
         <f>IF(OR(F25="",G25="",C25=""),"",(G25-F25)/F25*10000*IF(LOWER(C25)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I25" s="126" t="n"/>
+      <c r="I25" s="134" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="68">
-      <c r="A26" s="126" t="n"/>
-      <c r="B26" s="126" t="n"/>
-      <c r="C26" s="126" t="n"/>
-      <c r="D26" s="126" t="n"/>
+      <c r="A26" s="131" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B26" s="73" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C26" s="73" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D26" s="73" t="n">
+        <v>10.777954447</v>
+      </c>
       <c r="E26" s="78">
         <f>IF(OR(D26="",G26=""),"",D26*G26)</f>
         <v/>
       </c>
-      <c r="F26" s="125" t="n"/>
-      <c r="G26" s="125" t="n"/>
+      <c r="F26" s="78" t="n">
+        <v>717.1900000000001</v>
+      </c>
+      <c r="G26" s="78" t="n">
+        <v>717.088761</v>
+      </c>
       <c r="H26" s="135">
         <f>IF(OR(F26="",G26="",C26=""),"",(G26-F26)/F26*10000*IF(LOWER(C26)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I26" s="126" t="n"/>
+      <c r="I26" s="134" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="68">
       <c r="A27" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-16
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8104,7 +8104,7 @@
       <c r="G55" s="127" t="n">
         <v>340.980401015</v>
       </c>
-      <c r="H55" t="n">
+      <c r="H55" s="67" t="n">
         <v>73.81999999999999</v>
       </c>
       <c r="I55" s="84">
@@ -8216,8 +8216,12 @@
         <f>IF(AND(E56="",I56="",AE56="",AG56=""),"",SUM(E56,I56,AE56,AG56))</f>
         <v/>
       </c>
-      <c r="C56" s="119" t="n"/>
-      <c r="D56" s="84" t="n"/>
+      <c r="C56" s="119" t="n">
+        <v>106.861843804</v>
+      </c>
+      <c r="D56" s="84" t="n">
+        <v>709.8</v>
+      </c>
       <c r="E56" s="84">
         <f>IF(D56="","",D56*C56)</f>
         <v/>
@@ -8226,7 +8230,12 @@
         <f>IF(B56="","",E56/B56)</f>
         <v/>
       </c>
-      <c r="G56" s="127" t="n"/>
+      <c r="G56" s="127" t="n">
+        <v>420.916806674</v>
+      </c>
+      <c r="H56" t="n">
+        <v>68.20999999999999</v>
+      </c>
       <c r="I56" s="84">
         <f>IF(H56="","",H56*G56)</f>
         <v/>
@@ -8239,17 +8248,17 @@
         <f>IF(B56="","",F56+J56*3)</f>
         <v/>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="L56" s="67" t="inlineStr">
         <is>
           <t>1.57x</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="M56" s="67" t="inlineStr">
         <is>
           <t>REBALANCE — 76.83% QQQ / 23.17% TQQQ → 71.66% QQQ / 28.34% TQQQ</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="N56" s="67" t="inlineStr">
         <is>
           <t>1.57x</t>
         </is>
@@ -8266,15 +8275,15 @@
       <c r="R56" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S56" t="n">
+      <c r="S56" s="67" t="n">
         <v>133</v>
       </c>
-      <c r="T56" t="inlineStr">
+      <c r="T56" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="U56" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8317,8 +8326,14 @@
         <f>IF(OR(AE56="",B56="",B56=0),"",AE56/B56)</f>
         <v/>
       </c>
-      <c r="AG56" s="125" t="n"/>
-      <c r="AH56" s="126" t="n"/>
+      <c r="AG56" s="125" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="AH56" s="126" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="AI56" s="126" t="n"/>
       <c r="AJ56" s="126" t="n"/>
     </row>
@@ -8353,13 +8368,45 @@
         <f>IF(B57="","",F57+J57*3)</f>
         <v/>
       </c>
-      <c r="O57" s="122" t="n"/>
-      <c r="P57" s="83" t="n"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>1.38x</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>REBALANCE — 71.66% QQQ / 28.34% TQQQ → 81.16% QQQ / 18.84% TQQQ</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>1.38x</t>
+        </is>
+      </c>
+      <c r="O57" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P57" s="83" t="n">
+        <v>0.57</v>
+      </c>
       <c r="Q57" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R57" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S57" t="n">
+        <v>134</v>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V57" s="123">
         <f>IF(OR(B57="",B56=""),"",B57/B56-1)</f>
@@ -15487,38 +15534,70 @@
       <c r="I26" s="134" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="68">
-      <c r="A27" s="126" t="n"/>
-      <c r="B27" s="126" t="n"/>
-      <c r="C27" s="126" t="n"/>
-      <c r="D27" s="126" t="n"/>
+      <c r="A27" s="131" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B27" s="73" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C27" s="73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="D27" s="73" t="n">
+        <v>7.923060901</v>
+      </c>
       <c r="E27" s="78">
         <f>IF(OR(D27="",G27=""),"",D27*G27)</f>
         <v/>
       </c>
-      <c r="F27" s="125" t="n"/>
-      <c r="G27" s="125" t="n"/>
+      <c r="F27" s="78" t="n">
+        <v>720.205</v>
+      </c>
+      <c r="G27" s="78" t="n">
+        <v>720.1799999999999</v>
+      </c>
       <c r="H27" s="135">
         <f>IF(OR(F27="",G27="",C27=""),"",(G27-F27)/F27*10000*IF(LOWER(C27)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I27" s="126" t="n"/>
+      <c r="I27" s="134" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="68">
-      <c r="A28" s="126" t="n"/>
-      <c r="B28" s="126" t="n"/>
-      <c r="C28" s="126" t="n"/>
-      <c r="D28" s="126" t="n"/>
+      <c r="A28" s="131" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B28" s="73" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C28" s="73" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D28" s="73" t="n">
+        <v>79.936405659</v>
+      </c>
       <c r="E28" s="78">
         <f>IF(OR(D28="",G28=""),"",D28*G28)</f>
         <v/>
       </c>
-      <c r="F28" s="125" t="n"/>
-      <c r="G28" s="125" t="n"/>
+      <c r="F28" s="78" t="n">
+        <v>71.36499999999999</v>
+      </c>
+      <c r="G28" s="78" t="n">
+        <v>71.38199400000001</v>
+      </c>
       <c r="H28" s="135">
         <f>IF(OR(F28="",G28="",C28=""),"",(G28-F28)/F28*10000*IF(LOWER(C28)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I28" s="126" t="n"/>
+      <c r="I28" s="134" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="68">
       <c r="A29" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-19
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8233,7 +8233,7 @@
       <c r="G56" s="127" t="n">
         <v>420.916806674</v>
       </c>
-      <c r="H56" t="n">
+      <c r="H56" s="67" t="n">
         <v>68.20999999999999</v>
       </c>
       <c r="I56" s="84">
@@ -8345,8 +8345,12 @@
         <f>IF(AND(E57="",I57="",AE57="",AG57=""),"",SUM(E57,I57,AE57,AG57))</f>
         <v/>
       </c>
-      <c r="C57" s="119" t="n"/>
-      <c r="D57" s="84" t="n"/>
+      <c r="C57" s="119" t="n">
+        <v>120.458865998</v>
+      </c>
+      <c r="D57" s="84" t="n">
+        <v>718.36</v>
+      </c>
       <c r="E57" s="84">
         <f>IF(D57="","",D57*C57)</f>
         <v/>
@@ -8355,7 +8359,12 @@
         <f>IF(B57="","",E57/B57)</f>
         <v/>
       </c>
-      <c r="G57" s="127" t="n"/>
+      <c r="G57" s="127" t="n">
+        <v>282.904091218</v>
+      </c>
+      <c r="H57" t="n">
+        <v>70.64</v>
+      </c>
       <c r="I57" s="84">
         <f>IF(H57="","",H57*G57)</f>
         <v/>
@@ -8368,17 +8377,17 @@
         <f>IF(B57="","",F57+J57*3)</f>
         <v/>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L57" s="67" t="inlineStr">
         <is>
           <t>1.38x</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="M57" s="67" t="inlineStr">
         <is>
           <t>REBALANCE — 71.66% QQQ / 28.34% TQQQ → 81.16% QQQ / 18.84% TQQQ</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
+      <c r="N57" s="67" t="inlineStr">
         <is>
           <t>1.38x</t>
         </is>
@@ -8395,15 +8404,15 @@
       <c r="R57" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S57" t="n">
+      <c r="S57" s="67" t="n">
         <v>134</v>
       </c>
-      <c r="T57" t="inlineStr">
+      <c r="T57" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="U57" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8446,8 +8455,14 @@
         <f>IF(OR(AE57="",B57="",B57=0),"",AE57/B57)</f>
         <v/>
       </c>
-      <c r="AG57" s="125" t="n"/>
-      <c r="AH57" s="126" t="n"/>
+      <c r="AG57" s="125" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="AH57" s="126" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="AI57" s="126" t="n"/>
       <c r="AJ57" s="126" t="n"/>
     </row>
@@ -8482,13 +8497,45 @@
         <f>IF(B58="","",F58+J58*3)</f>
         <v/>
       </c>
-      <c r="O58" s="122" t="n"/>
-      <c r="P58" s="83" t="n"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>1.58x</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>REBALANCE — 81.16% QQQ / 18.84% TQQQ → 70.75% QQQ / 29.25% TQQQ</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>1.58x</t>
+        </is>
+      </c>
+      <c r="O58" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P58" s="83" t="n">
+        <v>0.58</v>
+      </c>
       <c r="Q58" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R58" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S58" t="n">
+        <v>135</v>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V58" s="123">
         <f>IF(OR(B58="",B57=""),"",B58/B57-1)</f>
@@ -15600,38 +15647,70 @@
       <c r="I28" s="134" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="68">
-      <c r="A29" s="126" t="n"/>
-      <c r="B29" s="126" t="n"/>
-      <c r="C29" s="126" t="n"/>
-      <c r="D29" s="126" t="n"/>
+      <c r="A29" s="131" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B29" s="73" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C29" s="73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="D29" s="73" t="n">
+        <v>138.012715456</v>
+      </c>
       <c r="E29" s="78">
         <f>IF(OR(D29="",G29=""),"",D29*G29)</f>
         <v/>
       </c>
-      <c r="F29" s="125" t="n"/>
-      <c r="G29" s="125" t="n"/>
+      <c r="F29" s="78" t="n">
+        <v>70.935</v>
+      </c>
+      <c r="G29" s="78" t="n">
+        <v>70.80014300000001</v>
+      </c>
       <c r="H29" s="135">
         <f>IF(OR(F29="",G29="",C29=""),"",(G29-F29)/F29*10000*IF(LOWER(C29)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I29" s="126" t="n"/>
+      <c r="I29" s="134" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="68">
-      <c r="A30" s="126" t="n"/>
-      <c r="B30" s="126" t="n"/>
-      <c r="C30" s="126" t="n"/>
-      <c r="D30" s="126" t="n"/>
+      <c r="A30" s="131" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B30" s="73" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C30" s="73" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D30" s="73" t="n">
+        <v>13.597022194</v>
+      </c>
       <c r="E30" s="78">
         <f>IF(OR(D30="",G30=""),"",D30*G30)</f>
         <v/>
       </c>
-      <c r="F30" s="125" t="n"/>
-      <c r="G30" s="125" t="n"/>
+      <c r="F30" s="78" t="n">
+        <v>719.34</v>
+      </c>
+      <c r="G30" s="78" t="n">
+        <v>718.716191</v>
+      </c>
       <c r="H30" s="135">
         <f>IF(OR(F30="",G30="",C30=""),"",(G30-F30)/F30*10000*IF(LOWER(C30)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I30" s="126" t="n"/>
+      <c r="I30" s="134" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="68">
       <c r="A31" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-20
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8362,7 +8362,7 @@
       <c r="G57" s="127" t="n">
         <v>282.904091218</v>
       </c>
-      <c r="H57" t="n">
+      <c r="H57" s="67" t="n">
         <v>70.64</v>
       </c>
       <c r="I57" s="84">
@@ -8474,8 +8474,12 @@
         <f>IF(AND(E58="",I58="",AE58="",AG58=""),"",SUM(E58,I58,AE58,AG58))</f>
         <v/>
       </c>
-      <c r="C58" s="119" t="n"/>
-      <c r="D58" s="84" t="n"/>
+      <c r="C58" s="119" t="n">
+        <v>104.841868283</v>
+      </c>
+      <c r="D58" s="84" t="n">
+        <v>717.63</v>
+      </c>
       <c r="E58" s="84">
         <f>IF(D58="","",D58*C58)</f>
         <v/>
@@ -8484,7 +8488,12 @@
         <f>IF(B58="","",E58/B58)</f>
         <v/>
       </c>
-      <c r="G58" s="127" t="n"/>
+      <c r="G58" s="127" t="n">
+        <v>444.008661654</v>
+      </c>
+      <c r="H58" t="n">
+        <v>70.41</v>
+      </c>
       <c r="I58" s="84">
         <f>IF(H58="","",H58*G58)</f>
         <v/>
@@ -8497,17 +8506,17 @@
         <f>IF(B58="","",F58+J58*3)</f>
         <v/>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L58" s="67" t="inlineStr">
         <is>
           <t>1.58x</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="M58" s="67" t="inlineStr">
         <is>
           <t>REBALANCE — 81.16% QQQ / 18.84% TQQQ → 70.75% QQQ / 29.25% TQQQ</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
+      <c r="N58" s="67" t="inlineStr">
         <is>
           <t>1.58x</t>
         </is>
@@ -8524,15 +8533,15 @@
       <c r="R58" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S58" t="n">
+      <c r="S58" s="67" t="n">
         <v>135</v>
       </c>
-      <c r="T58" t="inlineStr">
+      <c r="T58" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="U58" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8575,8 +8584,14 @@
         <f>IF(OR(AE58="",B58="",B58=0),"",AE58/B58)</f>
         <v/>
       </c>
-      <c r="AG58" s="125" t="n"/>
-      <c r="AH58" s="126" t="n"/>
+      <c r="AG58" s="125" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="AH58" s="126" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="AI58" s="126" t="n"/>
       <c r="AJ58" s="126" t="n"/>
     </row>
@@ -8611,13 +8626,45 @@
         <f>IF(B59="","",F59+J59*3)</f>
         <v/>
       </c>
-      <c r="O59" s="122" t="n"/>
-      <c r="P59" s="83" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>1.58x</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>1.61x</t>
+        </is>
+      </c>
+      <c r="O59" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P59" s="83" t="n">
+        <v>0.58</v>
+      </c>
       <c r="Q59" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R59" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S59" t="n">
+        <v>136</v>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V59" s="123">
         <f>IF(OR(B59="",B58=""),"",B59/B58-1)</f>
@@ -15713,38 +15760,70 @@
       <c r="I30" s="134" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="68">
-      <c r="A31" s="126" t="n"/>
-      <c r="B31" s="126" t="n"/>
-      <c r="C31" s="126" t="n"/>
-      <c r="D31" s="126" t="n"/>
+      <c r="A31" s="131" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B31" s="73" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C31" s="73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="D31" s="73" t="n">
+        <v>15.616997715</v>
+      </c>
       <c r="E31" s="78">
         <f>IF(OR(D31="",G31=""),"",D31*G31)</f>
         <v/>
       </c>
-      <c r="F31" s="125" t="n"/>
-      <c r="G31" s="125" t="n"/>
+      <c r="F31" s="78" t="n">
+        <v>713.535</v>
+      </c>
+      <c r="G31" s="78" t="n">
+        <v>713.4521120000001</v>
+      </c>
       <c r="H31" s="135">
         <f>IF(OR(F31="",G31="",C31=""),"",(G31-F31)/F31*10000*IF(LOWER(C31)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I31" s="126" t="n"/>
+      <c r="I31" s="134" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="68">
-      <c r="A32" s="126" t="n"/>
-      <c r="B32" s="126" t="n"/>
-      <c r="C32" s="126" t="n"/>
-      <c r="D32" s="126" t="n"/>
+      <c r="A32" s="131" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B32" s="73" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C32" s="73" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D32" s="73" t="n">
+        <v>161.104570436</v>
+      </c>
       <c r="E32" s="78">
         <f>IF(OR(D32="",G32=""),"",D32*G32)</f>
         <v/>
       </c>
-      <c r="F32" s="125" t="n"/>
-      <c r="G32" s="125" t="n"/>
+      <c r="F32" s="78" t="n">
+        <v>69.215</v>
+      </c>
+      <c r="G32" s="78" t="n">
+        <v>69.178359</v>
+      </c>
       <c r="H32" s="135">
         <f>IF(OR(F32="",G32="",C32=""),"",(G32-F32)/F32*10000*IF(LOWER(C32)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I32" s="126" t="n"/>
+      <c r="I32" s="134" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="68">
       <c r="A33" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-21
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8491,7 +8491,7 @@
       <c r="G58" s="127" t="n">
         <v>444.008661654</v>
       </c>
-      <c r="H58" t="n">
+      <c r="H58" s="67" t="n">
         <v>70.41</v>
       </c>
       <c r="I58" s="84">
@@ -8603,8 +8603,12 @@
         <f>IF(AND(E59="",I59="",AE59="",AG59=""),"",SUM(E59,I59,AE59,AG59))</f>
         <v/>
       </c>
-      <c r="C59" s="119" t="n"/>
-      <c r="D59" s="84" t="n"/>
+      <c r="C59" s="119" t="n">
+        <v>104.841868283</v>
+      </c>
+      <c r="D59" s="84" t="n">
+        <v>725.2</v>
+      </c>
       <c r="E59" s="84">
         <f>IF(D59="","",D59*C59)</f>
         <v/>
@@ -8613,7 +8617,12 @@
         <f>IF(B59="","",E59/B59)</f>
         <v/>
       </c>
-      <c r="G59" s="127" t="n"/>
+      <c r="G59" s="127" t="n">
+        <v>444.008661654</v>
+      </c>
+      <c r="H59" t="n">
+        <v>72.61</v>
+      </c>
       <c r="I59" s="84">
         <f>IF(H59="","",H59*G59)</f>
         <v/>
@@ -8626,17 +8635,17 @@
         <f>IF(B59="","",F59+J59*3)</f>
         <v/>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="L59" s="67" t="inlineStr">
         <is>
           <t>1.58x</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="M59" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
+      <c r="N59" s="67" t="inlineStr">
         <is>
           <t>1.61x</t>
         </is>
@@ -8653,15 +8662,15 @@
       <c r="R59" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S59" t="n">
+      <c r="S59" s="67" t="n">
         <v>136</v>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="T59" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="U59" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8704,7 +8713,9 @@
         <f>IF(OR(AE59="",B59="",B59=0),"",AE59/B59)</f>
         <v/>
       </c>
-      <c r="AG59" s="125" t="n"/>
+      <c r="AG59" s="125" t="n">
+        <v>-4.81</v>
+      </c>
       <c r="AH59" s="126" t="n"/>
       <c r="AI59" s="126" t="n"/>
       <c r="AJ59" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-22
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8620,7 +8620,7 @@
       <c r="G59" s="127" t="n">
         <v>444.008661654</v>
       </c>
-      <c r="H59" t="n">
+      <c r="H59" s="67" t="n">
         <v>72.61</v>
       </c>
       <c r="I59" s="84">
@@ -8728,8 +8728,12 @@
         <f>IF(AND(E60="",I60="",AE60="",AG60=""),"",SUM(E60,I60,AE60,AG60))</f>
         <v/>
       </c>
-      <c r="C60" s="119" t="n"/>
-      <c r="D60" s="84" t="n"/>
+      <c r="C60" s="119" t="n">
+        <v>104.841868283</v>
+      </c>
+      <c r="D60" s="84" t="n">
+        <v>704.47</v>
+      </c>
       <c r="E60" s="84">
         <f>IF(D60="","",D60*C60)</f>
         <v/>
@@ -8738,7 +8742,12 @@
         <f>IF(B60="","",E60/B60)</f>
         <v/>
       </c>
-      <c r="G60" s="127" t="n"/>
+      <c r="G60" s="127" t="n">
+        <v>444.008661654</v>
+      </c>
+      <c r="H60" t="n">
+        <v>66.42</v>
+      </c>
       <c r="I60" s="84">
         <f>IF(H60="","",H60*G60)</f>
         <v/>
@@ -8797,7 +8806,9 @@
         <f>IF(OR(AE60="",B60="",B60=0),"",AE60/B60)</f>
         <v/>
       </c>
-      <c r="AG60" s="125" t="n"/>
+      <c r="AG60" s="125" t="n">
+        <v>-4.81</v>
+      </c>
       <c r="AH60" s="126" t="n"/>
       <c r="AI60" s="126" t="n"/>
       <c r="AJ60" s="126" t="n"/>
@@ -8833,13 +8844,45 @@
         <f>IF(B61="","",F61+J61*3)</f>
         <v/>
       </c>
-      <c r="O61" s="122" t="n"/>
-      <c r="P61" s="83" t="n"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>REBALANCE — 70.75% QQQ / 29.25% TQQQ → 83.75% QQQ / 16.25% TQQQ</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="O61" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P61" s="83" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="Q61" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R61" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S61" t="n">
+        <v>138</v>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V61" s="123">
         <f>IF(OR(B61="",B60=""),"",B61/B60-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-23
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8745,7 +8745,7 @@
       <c r="G60" s="127" t="n">
         <v>444.008661654</v>
       </c>
-      <c r="H60" t="n">
+      <c r="H60" s="67" t="n">
         <v>66.42</v>
       </c>
       <c r="I60" s="84">
@@ -8760,13 +8760,45 @@
         <f>IF(B60="","",F60+J60*3)</f>
         <v/>
       </c>
-      <c r="O60" s="122" t="n"/>
-      <c r="P60" s="83" t="n"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>1.58x</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>1.59x</t>
+        </is>
+      </c>
+      <c r="O60" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P60" s="83" t="n">
+        <v>0.52</v>
+      </c>
       <c r="Q60" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R60" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S60" t="n">
+        <v>137</v>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V60" s="123">
         <f>IF(OR(B60="",B59=""),"",B60/B59-1)</f>
@@ -8821,8 +8853,12 @@
         <f>IF(AND(E61="",I61="",AE61="",AG61=""),"",SUM(E61,I61,AE61,AG61))</f>
         <v/>
       </c>
-      <c r="C61" s="119" t="n"/>
-      <c r="D61" s="84" t="n"/>
+      <c r="C61" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D61" s="84" t="n">
+        <v>704.4</v>
+      </c>
       <c r="E61" s="84">
         <f>IF(D61="","",D61*C61)</f>
         <v/>
@@ -8831,7 +8867,12 @@
         <f>IF(B61="","",E61/B61)</f>
         <v/>
       </c>
-      <c r="G61" s="127" t="n"/>
+      <c r="G61" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H61" t="n">
+        <v>66.29000000000001</v>
+      </c>
       <c r="I61" s="84">
         <f>IF(H61="","",H61*G61)</f>
         <v/>
@@ -8844,17 +8885,17 @@
         <f>IF(B61="","",F61+J61*3)</f>
         <v/>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="L61" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="M61" s="67" t="inlineStr">
         <is>
           <t>REBALANCE — 70.75% QQQ / 29.25% TQQQ → 83.75% QQQ / 16.25% TQQQ</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
+      <c r="N61" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
@@ -8871,15 +8912,15 @@
       <c r="R61" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S61" t="n">
+      <c r="S61" s="67" t="n">
         <v>138</v>
       </c>
-      <c r="T61" t="inlineStr">
+      <c r="T61" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="U61" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8922,8 +8963,14 @@
         <f>IF(OR(AE61="",B61="",B61=0),"",AE61/B61)</f>
         <v/>
       </c>
-      <c r="AG61" s="125" t="n"/>
-      <c r="AH61" s="126" t="n"/>
+      <c r="AG61" s="125" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AH61" s="126" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="AI61" s="126" t="n"/>
       <c r="AJ61" s="126" t="n"/>
     </row>
@@ -8958,13 +9005,45 @@
         <f>IF(B62="","",F62+J62*3)</f>
         <v/>
       </c>
-      <c r="O62" s="122" t="n"/>
-      <c r="P62" s="83" t="n"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>1.33x</t>
+        </is>
+      </c>
+      <c r="O62" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P62" s="83" t="n">
+        <v>0.57</v>
+      </c>
       <c r="Q62" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R62" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S62" t="n">
+        <v>139</v>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V62" s="123">
         <f>IF(OR(B62="",B61=""),"",B62/B61-1)</f>
@@ -15880,38 +15959,70 @@
       <c r="I32" s="134" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="68">
-      <c r="A33" s="126" t="n"/>
-      <c r="B33" s="126" t="n"/>
-      <c r="C33" s="126" t="n"/>
-      <c r="D33" s="126" t="n"/>
+      <c r="A33" s="131" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B33" s="73" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C33" s="73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="D33" s="73" t="n">
+        <v>193.075324675</v>
+      </c>
       <c r="E33" s="78">
         <f>IF(OR(D33="",G33=""),"",D33*G33)</f>
         <v/>
       </c>
-      <c r="F33" s="125" t="n"/>
-      <c r="G33" s="125" t="n"/>
+      <c r="F33" s="78" t="n">
+        <v>65.47499999999999</v>
+      </c>
+      <c r="G33" s="78" t="n">
+        <v>65.45300400000001</v>
+      </c>
       <c r="H33" s="135">
         <f>IF(OR(F33="",G33="",C33=""),"",(G33-F33)/F33*10000*IF(LOWER(C33)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I33" s="126" t="n"/>
+      <c r="I33" s="134" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="68">
-      <c r="A34" s="126" t="n"/>
-      <c r="B34" s="126" t="n"/>
-      <c r="C34" s="126" t="n"/>
-      <c r="D34" s="126" t="n"/>
+      <c r="A34" s="131" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B34" s="73" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C34" s="73" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D34" s="73" t="n">
+        <v>18.008753296</v>
+      </c>
       <c r="E34" s="78">
         <f>IF(OR(D34="",G34=""),"",D34*G34)</f>
         <v/>
       </c>
-      <c r="F34" s="125" t="n"/>
-      <c r="G34" s="125" t="n"/>
+      <c r="F34" s="78" t="n">
+        <v>701.495</v>
+      </c>
+      <c r="G34" s="78" t="n">
+        <v>701.467214</v>
+      </c>
       <c r="H34" s="135">
         <f>IF(OR(F34="",G34="",C34=""),"",(G34-F34)/F34*10000*IF(LOWER(C34)="buy",1,-1))</f>
         <v/>
       </c>
-      <c r="I34" s="126" t="n"/>
+      <c r="I34" s="134" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="68">
       <c r="A35" s="126" t="n"/>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-26
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8760,17 +8760,17 @@
         <f>IF(B60="","",F60+J60*3)</f>
         <v/>
       </c>
-      <c r="L60" t="inlineStr">
+      <c r="L60" s="67" t="inlineStr">
         <is>
           <t>1.58x</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="M60" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
+      <c r="N60" s="67" t="inlineStr">
         <is>
           <t>1.59x</t>
         </is>
@@ -8787,15 +8787,15 @@
       <c r="R60" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S60" t="n">
+      <c r="S60" s="67" t="n">
         <v>137</v>
       </c>
-      <c r="T60" t="inlineStr">
+      <c r="T60" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="U60" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8870,7 +8870,7 @@
       <c r="G61" s="127" t="n">
         <v>250.933336979</v>
       </c>
-      <c r="H61" t="n">
+      <c r="H61" s="67" t="n">
         <v>66.29000000000001</v>
       </c>
       <c r="I61" s="84">
@@ -8964,7 +8964,7 @@
         <v/>
       </c>
       <c r="AG61" s="125" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AH61" s="126" t="inlineStr">
         <is>
@@ -8982,8 +8982,12 @@
         <f>IF(AND(E62="",I62="",AE62="",AG62=""),"",SUM(E62,I62,AE62,AG62))</f>
         <v/>
       </c>
-      <c r="C62" s="119" t="n"/>
-      <c r="D62" s="84" t="n"/>
+      <c r="C62" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D62" s="84" t="n">
+        <v>712.2</v>
+      </c>
       <c r="E62" s="84">
         <f>IF(D62="","",D62*C62)</f>
         <v/>
@@ -8992,7 +8996,12 @@
         <f>IF(B62="","",E62/B62)</f>
         <v/>
       </c>
-      <c r="G62" s="127" t="n"/>
+      <c r="G62" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H62" t="n">
+        <v>68.43000000000001</v>
+      </c>
       <c r="I62" s="84">
         <f>IF(H62="","",H62*G62)</f>
         <v/>
@@ -9005,17 +9014,17 @@
         <f>IF(B62="","",F62+J62*3)</f>
         <v/>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L62" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="M62" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="N62" s="67" t="inlineStr">
         <is>
           <t>1.33x</t>
         </is>
@@ -9032,15 +9041,15 @@
       <c r="R62" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S62" t="n">
+      <c r="S62" s="67" t="n">
         <v>139</v>
       </c>
-      <c r="T62" t="inlineStr">
+      <c r="T62" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="U62" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -9083,7 +9092,9 @@
         <f>IF(OR(AE62="",B62="",B62=0),"",AE62/B62)</f>
         <v/>
       </c>
-      <c r="AG62" s="125" t="n"/>
+      <c r="AG62" s="125" t="n">
+        <v>-0.28</v>
+      </c>
       <c r="AH62" s="126" t="n"/>
       <c r="AI62" s="126" t="n"/>
       <c r="AJ62" s="126" t="n"/>
@@ -9119,13 +9130,45 @@
         <f>IF(B63="","",F63+J63*3)</f>
         <v/>
       </c>
-      <c r="O63" s="122" t="n"/>
-      <c r="P63" s="83" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>1.33x</t>
+        </is>
+      </c>
+      <c r="O63" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P63" s="83" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="Q63" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R63" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S63" t="n">
+        <v>140</v>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V63" s="123">
         <f>IF(OR(B63="",B62=""),"",B63/B62-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-27
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -8999,7 +8999,7 @@
       <c r="G62" s="127" t="n">
         <v>250.933336979</v>
       </c>
-      <c r="H62" t="n">
+      <c r="H62" s="67" t="n">
         <v>68.43000000000001</v>
       </c>
       <c r="I62" s="84">
@@ -9107,8 +9107,12 @@
         <f>IF(AND(E63="",I63="",AE63="",AG63=""),"",SUM(E63,I63,AE63,AG63))</f>
         <v/>
       </c>
-      <c r="C63" s="119" t="n"/>
-      <c r="D63" s="84" t="n"/>
+      <c r="C63" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D63" s="84" t="n">
+        <v>721.25</v>
+      </c>
       <c r="E63" s="84">
         <f>IF(D63="","",D63*C63)</f>
         <v/>
@@ -9117,7 +9121,12 @@
         <f>IF(B63="","",E63/B63)</f>
         <v/>
       </c>
-      <c r="G63" s="127" t="n"/>
+      <c r="G63" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H63" t="n">
+        <v>71.04000000000001</v>
+      </c>
       <c r="I63" s="84">
         <f>IF(H63="","",H63*G63)</f>
         <v/>
@@ -9130,17 +9139,17 @@
         <f>IF(B63="","",F63+J63*3)</f>
         <v/>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L63" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="M63" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="N63" s="67" t="inlineStr">
         <is>
           <t>1.33x</t>
         </is>
@@ -9157,15 +9166,15 @@
       <c r="R63" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S63" t="n">
+      <c r="S63" s="67" t="n">
         <v>140</v>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="T63" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="U63" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -9208,7 +9217,9 @@
         <f>IF(OR(AE63="",B63="",B63=0),"",AE63/B63)</f>
         <v/>
       </c>
-      <c r="AG63" s="125" t="n"/>
+      <c r="AG63" s="125" t="n">
+        <v>-0.28</v>
+      </c>
       <c r="AH63" s="126" t="n"/>
       <c r="AI63" s="126" t="n"/>
       <c r="AJ63" s="126" t="n"/>
@@ -9244,13 +9255,45 @@
         <f>IF(B64="","",F64+J64*3)</f>
         <v/>
       </c>
-      <c r="O64" s="122" t="n"/>
-      <c r="P64" s="83" t="n"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>1.29x</t>
+        </is>
+      </c>
+      <c r="O64" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P64" s="83" t="n">
+        <v>0.54</v>
+      </c>
       <c r="Q64" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R64" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S64" t="n">
+        <v>141</v>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V64" s="123">
         <f>IF(OR(B64="",B63=""),"",B64/B63-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-28
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -9124,7 +9124,7 @@
       <c r="G63" s="127" t="n">
         <v>250.933336979</v>
       </c>
-      <c r="H63" t="n">
+      <c r="H63" s="67" t="n">
         <v>71.04000000000001</v>
       </c>
       <c r="I63" s="84">
@@ -9232,8 +9232,12 @@
         <f>IF(AND(E64="",I64="",AE64="",AG64=""),"",SUM(E64,I64,AE64,AG64))</f>
         <v/>
       </c>
-      <c r="C64" s="119" t="n"/>
-      <c r="D64" s="84" t="n"/>
+      <c r="C64" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D64" s="84" t="n">
+        <v>725.61</v>
+      </c>
       <c r="E64" s="84">
         <f>IF(D64="","",D64*C64)</f>
         <v/>
@@ -9242,7 +9246,12 @@
         <f>IF(B64="","",E64/B64)</f>
         <v/>
       </c>
-      <c r="G64" s="127" t="n"/>
+      <c r="G64" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H64" t="n">
+        <v>72.36</v>
+      </c>
       <c r="I64" s="84">
         <f>IF(H64="","",H64*G64)</f>
         <v/>
@@ -9255,17 +9264,17 @@
         <f>IF(B64="","",F64+J64*3)</f>
         <v/>
       </c>
-      <c r="L64" t="inlineStr">
+      <c r="L64" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="M64" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
+      <c r="N64" s="67" t="inlineStr">
         <is>
           <t>1.29x</t>
         </is>
@@ -9282,15 +9291,15 @@
       <c r="R64" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S64" t="n">
+      <c r="S64" s="67" t="n">
         <v>141</v>
       </c>
-      <c r="T64" t="inlineStr">
+      <c r="T64" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="U64" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -9333,7 +9342,9 @@
         <f>IF(OR(AE64="",B64="",B64=0),"",AE64/B64)</f>
         <v/>
       </c>
-      <c r="AG64" s="125" t="n"/>
+      <c r="AG64" s="125" t="n">
+        <v>-0.28</v>
+      </c>
       <c r="AH64" s="126" t="n"/>
       <c r="AI64" s="126" t="n"/>
       <c r="AJ64" s="126" t="n"/>
@@ -9369,13 +9380,45 @@
         <f>IF(B65="","",F65+J65*3)</f>
         <v/>
       </c>
-      <c r="O65" s="122" t="n"/>
-      <c r="P65" s="83" t="n"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>1.29x</t>
+        </is>
+      </c>
+      <c r="O65" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P65" s="83" t="n">
+        <v>0.54</v>
+      </c>
       <c r="Q65" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R65" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S65" t="n">
+        <v>142</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V65" s="123">
         <f>IF(OR(B65="",B64=""),"",B65/B64-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-29
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -9249,7 +9249,7 @@
       <c r="G64" s="127" t="n">
         <v>250.933336979</v>
       </c>
-      <c r="H64" t="n">
+      <c r="H64" s="67" t="n">
         <v>72.36</v>
       </c>
       <c r="I64" s="84">
@@ -9357,8 +9357,12 @@
         <f>IF(AND(E65="",I65="",AE65="",AG65=""),"",SUM(E65,I65,AE65,AG65))</f>
         <v/>
       </c>
-      <c r="C65" s="119" t="n"/>
-      <c r="D65" s="84" t="n"/>
+      <c r="C65" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D65" s="84" t="n">
+        <v>715.34</v>
+      </c>
       <c r="E65" s="84">
         <f>IF(D65="","",D65*C65)</f>
         <v/>
@@ -9367,7 +9371,12 @@
         <f>IF(B65="","",E65/B65)</f>
         <v/>
       </c>
-      <c r="G65" s="127" t="n"/>
+      <c r="G65" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H65" t="n">
+        <v>69.26000000000001</v>
+      </c>
       <c r="I65" s="84">
         <f>IF(H65="","",H65*G65)</f>
         <v/>
@@ -9380,17 +9389,17 @@
         <f>IF(B65="","",F65+J65*3)</f>
         <v/>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L65" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="M65" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
+      <c r="N65" s="67" t="inlineStr">
         <is>
           <t>1.29x</t>
         </is>
@@ -9407,15 +9416,15 @@
       <c r="R65" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S65" t="n">
+      <c r="S65" s="67" t="n">
         <v>142</v>
       </c>
-      <c r="T65" t="inlineStr">
+      <c r="T65" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="U65" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -9458,7 +9467,9 @@
         <f>IF(OR(AE65="",B65="",B65=0),"",AE65/B65)</f>
         <v/>
       </c>
-      <c r="AG65" s="125" t="n"/>
+      <c r="AG65" s="125" t="n">
+        <v>-0.28</v>
+      </c>
       <c r="AH65" s="126" t="n"/>
       <c r="AI65" s="126" t="n"/>
       <c r="AJ65" s="126" t="n"/>
@@ -9494,13 +9505,45 @@
         <f>IF(B66="","",F66+J66*3)</f>
         <v/>
       </c>
-      <c r="O66" s="122" t="n"/>
-      <c r="P66" s="83" t="n"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>1.32x</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>no change - hold current position</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>1.25x</t>
+        </is>
+      </c>
+      <c r="O66" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P66" s="83" t="n">
+        <v>0.55</v>
+      </c>
       <c r="Q66" s="83" t="n">
         <v>0.91</v>
       </c>
       <c r="R66" s="83" t="n">
         <v>0.37</v>
+      </c>
+      <c r="S66" t="n">
+        <v>143</v>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="V66" s="123">
         <f>IF(OR(B66="",B65=""),"",B66/B65-1)</f>

</xml_diff>

<commit_message>
Update v3.3 ledger 2026-10-30
</commit_message>
<xml_diff>
--- a/ledger/v33_paper_trading.xlsx
+++ b/ledger/v33_paper_trading.xlsx
@@ -9374,7 +9374,7 @@
       <c r="G65" s="127" t="n">
         <v>250.933336979</v>
       </c>
-      <c r="H65" t="n">
+      <c r="H65" s="67" t="n">
         <v>69.26000000000001</v>
       </c>
       <c r="I65" s="84">
@@ -9482,8 +9482,12 @@
         <f>IF(AND(E66="",I66="",AE66="",AG66=""),"",SUM(E66,I66,AE66,AG66))</f>
         <v/>
       </c>
-      <c r="C66" s="119" t="n"/>
-      <c r="D66" s="84" t="n"/>
+      <c r="C66" s="119" t="n">
+        <v>122.850621579</v>
+      </c>
+      <c r="D66" s="84" t="n">
+        <v>690.49</v>
+      </c>
       <c r="E66" s="84">
         <f>IF(D66="","",D66*C66)</f>
         <v/>
@@ -9492,7 +9496,12 @@
         <f>IF(B66="","",E66/B66)</f>
         <v/>
       </c>
-      <c r="G66" s="127" t="n"/>
+      <c r="G66" s="127" t="n">
+        <v>250.933336979</v>
+      </c>
+      <c r="H66" t="n">
+        <v>62.01</v>
+      </c>
       <c r="I66" s="84">
         <f>IF(H66="","",H66*G66)</f>
         <v/>
@@ -9505,17 +9514,17 @@
         <f>IF(B66="","",F66+J66*3)</f>
         <v/>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L66" s="67" t="inlineStr">
         <is>
           <t>1.32x</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="M66" s="67" t="inlineStr">
         <is>
           <t>no change - hold current position</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr">
+      <c r="N66" s="67" t="inlineStr">
         <is>
           <t>1.25x</t>
         </is>
@@ -9532,15 +9541,15 @@
       <c r="R66" s="83" t="n">
         <v>0.37</v>
       </c>
-      <c r="S66" t="n">
+      <c r="S66" s="67" t="n">
         <v>143</v>
       </c>
-      <c r="T66" t="inlineStr">
+      <c r="T66" s="67" t="inlineStr">
         <is>
           <t>above</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="U66" s="67" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -9583,7 +9592,9 @@
         <f>IF(OR(AE66="",B66="",B66=0),"",AE66/B66)</f>
         <v/>
       </c>
-      <c r="AG66" s="125" t="n"/>
+      <c r="AG66" s="125" t="n">
+        <v>-0.28</v>
+      </c>
       <c r="AH66" s="126" t="n"/>
       <c r="AI66" s="126" t="n"/>
       <c r="AJ66" s="126" t="n"/>
@@ -9619,10 +9630,46 @@
         <f>IF(B67="","",F67+J67*3)</f>
         <v/>
       </c>
-      <c r="O67" s="122" t="n"/>
-      <c r="P67" s="83" t="n"/>
-      <c r="Q67" s="83" t="n"/>
-      <c r="R67" s="83" t="n"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>1.00x</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>REBALANCE — 83.75% QQQ / 16.25% TQQQ → 100% QQQ</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>1.07x</t>
+        </is>
+      </c>
+      <c r="O67" s="122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="P67" s="83" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="Q67" s="83" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="R67" s="83" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="S67" t="n">
+        <v>144</v>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>above</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="V67" s="123">
         <f>IF(OR(B67="",B66=""),"",B67/B66-1)</f>
         <v/>

</xml_diff>